<commit_message>
Coral cove AMR export added
</commit_message>
<xml_diff>
--- a/ZLM_AMR_Export_2026-10-05.xlsx
+++ b/ZLM_AMR_Export_2026-10-05.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Temp folders/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Zululami/Site Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{556B839D-E021-47C5-9D2A-D125AC64FADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{556B839D-E021-47C5-9D2A-D125AC64FADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1474863D-B1E6-4348-AA74-0CCDA3B4CFD8}"/>
   <bookViews>
-    <workbookView xWindow="88080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{560B4A97-73D2-4BFB-BEAC-34EBBBAAD24C}"/>
+    <workbookView xWindow="59280" yWindow="-2430" windowWidth="29040" windowHeight="15720" xr2:uid="{560B4A97-73D2-4BFB-BEAC-34EBBBAAD24C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="587">
   <si>
     <t>SNR</t>
   </si>
@@ -732,6 +732,1074 @@
   </si>
   <si>
     <t>16816.001 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641067ff_5</t>
+  </si>
+  <si>
+    <t>Coral Cove 176 [Elec]</t>
+  </si>
+  <si>
+    <t>9/22/2026, 03:44 PM</t>
+  </si>
+  <si>
+    <t>4.633 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641067ff_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 177 [Elec]</t>
+  </si>
+  <si>
+    <t>9/22/2026, 03:43 PM</t>
+  </si>
+  <si>
+    <t>44.156 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641067ff_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 181 [Elec]</t>
+  </si>
+  <si>
+    <t>21.785 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641067ff_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 175 [Elec]</t>
+  </si>
+  <si>
+    <t>65.007 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641067ff_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 178 [Elec]</t>
+  </si>
+  <si>
+    <t>60.592 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641066ca_5</t>
+  </si>
+  <si>
+    <t>Coral Cove 106 [Elec]</t>
+  </si>
+  <si>
+    <t>9/29/2026, 04:28 PM</t>
+  </si>
+  <si>
+    <t>376.841 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641066ca_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 105 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:44 AM</t>
+  </si>
+  <si>
+    <t>1077.993 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641066ca_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 104 [Elec]</t>
+  </si>
+  <si>
+    <t>1688.322 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641066ca_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 103 [Elec]</t>
+  </si>
+  <si>
+    <t>613.253 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641066ca_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 75 [Elec]</t>
+  </si>
+  <si>
+    <t>564.607 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641060c2_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 155 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 09:16 AM</t>
+  </si>
+  <si>
+    <t>115.645 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641060c2_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 154 [Elec]</t>
+  </si>
+  <si>
+    <t>131.005 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641060c2_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 136 [Elec]</t>
+  </si>
+  <si>
+    <t>1335.962 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120641060c2_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 135 [Elec]</t>
+  </si>
+  <si>
+    <t>819.604 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105bd5_4</t>
+  </si>
+  <si>
+    <t>Coral Cove B001 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:49 AM</t>
+  </si>
+  <si>
+    <t>1556.503 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105bd5_3</t>
+  </si>
+  <si>
+    <t>Coral Cove B002 [Elec]</t>
+  </si>
+  <si>
+    <t>1021.623 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105bd5_2</t>
+  </si>
+  <si>
+    <t>Coral Cove B003 [Elec]</t>
+  </si>
+  <si>
+    <t>1395.043 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105bd5_1</t>
+  </si>
+  <si>
+    <t>Coral Cove B004 [Elec]</t>
+  </si>
+  <si>
+    <t>1853.518 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105981_6</t>
+  </si>
+  <si>
+    <t>Coral Cove 186 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 09:26 AM</t>
+  </si>
+  <si>
+    <t>679.917 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105981_5</t>
+  </si>
+  <si>
+    <t>Coral Cove 191 [Elec]</t>
+  </si>
+  <si>
+    <t>361.122 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105981_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 190 [Elec]</t>
+  </si>
+  <si>
+    <t>10/1/2026, 12:19 PM</t>
+  </si>
+  <si>
+    <t>186.055 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105981_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 188 [Elec]</t>
+  </si>
+  <si>
+    <t>130.349 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105981_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 187 [Elec]</t>
+  </si>
+  <si>
+    <t>1468.303 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105981_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 1xx [Elec]</t>
+  </si>
+  <si>
+    <t>91732851xx</t>
+  </si>
+  <si>
+    <t>516.123 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105970_4</t>
+  </si>
+  <si>
+    <t>Coral Cove B104 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 07:52 AM</t>
+  </si>
+  <si>
+    <t>1609.862 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105970_3</t>
+  </si>
+  <si>
+    <t>Coral Cove B103 [Elec]</t>
+  </si>
+  <si>
+    <t>586.02 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105970_2</t>
+  </si>
+  <si>
+    <t>Coral Cove B102 [Elec]</t>
+  </si>
+  <si>
+    <t>1495.716 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105970_1</t>
+  </si>
+  <si>
+    <t>Coral Cove B101 [Elec]</t>
+  </si>
+  <si>
+    <t>1298.523 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105879_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 66 [Elec]</t>
+  </si>
+  <si>
+    <t>6/12/2026, 03:03 PM</t>
+  </si>
+  <si>
+    <t>1723.497 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105879_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 65 [Elec]</t>
+  </si>
+  <si>
+    <t>184.281 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105879_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 64 [Elec]</t>
+  </si>
+  <si>
+    <t>1814.047 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105742_5</t>
+  </si>
+  <si>
+    <t>Coral Cove A105 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 09:06 AM</t>
+  </si>
+  <si>
+    <t>754.997 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105742_4</t>
+  </si>
+  <si>
+    <t>Coral Cove A104 [Elec]</t>
+  </si>
+  <si>
+    <t>1898.778 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105742_3</t>
+  </si>
+  <si>
+    <t>Coral Cove A103 [Elec]</t>
+  </si>
+  <si>
+    <t>1287.982 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105742_2</t>
+  </si>
+  <si>
+    <t>Coral Cove A102 [Elec]</t>
+  </si>
+  <si>
+    <t>1257.434 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105742_1</t>
+  </si>
+  <si>
+    <t>Coral Cove A101 [Elec]</t>
+  </si>
+  <si>
+    <t>2673.314 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105678_9</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 1</t>
+  </si>
+  <si>
+    <t>10/9/2026, 07:49 AM</t>
+  </si>
+  <si>
+    <t>45.219 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105678_8</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 2</t>
+  </si>
+  <si>
+    <t>139.166 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105678_7</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 3</t>
+  </si>
+  <si>
+    <t>154.66 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105678_6</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 4</t>
+  </si>
+  <si>
+    <t>168.91 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105678_5</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 14</t>
+  </si>
+  <si>
+    <t>97.667 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105678_4</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 15</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:53 AM</t>
+  </si>
+  <si>
+    <t>84.615 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105678_3</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 16</t>
+  </si>
+  <si>
+    <t>75.714 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105678_2</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 17</t>
+  </si>
+  <si>
+    <t>160.516 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064105678_1</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 18</t>
+  </si>
+  <si>
+    <t>191.352 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064104e86_5</t>
+  </si>
+  <si>
+    <t>Coral Cove A001 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 09:09 AM</t>
+  </si>
+  <si>
+    <t>1260.172 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064104e86_4</t>
+  </si>
+  <si>
+    <t>Coral Cove A002 [Elec]</t>
+  </si>
+  <si>
+    <t>879.187 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064104e86_3</t>
+  </si>
+  <si>
+    <t>Coral Cove A003 [Elec]</t>
+  </si>
+  <si>
+    <t>1166.201 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064104e86_2</t>
+  </si>
+  <si>
+    <t>Coral Cove A004 [Elec]</t>
+  </si>
+  <si>
+    <t>1240.541 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12064104e86_1</t>
+  </si>
+  <si>
+    <t>Coral Cove A005 [Elec]</t>
+  </si>
+  <si>
+    <t>1512.324 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635025eb_6</t>
+  </si>
+  <si>
+    <t>Coral Cove 72 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 09:13 AM</t>
+  </si>
+  <si>
+    <t>472.954 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635025eb_5</t>
+  </si>
+  <si>
+    <t>Coral Cove 71 [Elec]</t>
+  </si>
+  <si>
+    <t>376.124 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635025eb_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 70 [Elec]</t>
+  </si>
+  <si>
+    <t>994.387 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635025eb_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 69 [Elec]</t>
+  </si>
+  <si>
+    <t>1414.72 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635025eb_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 68 [Elec]</t>
+  </si>
+  <si>
+    <t>312.255 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635025eb_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 67 [Elec]</t>
+  </si>
+  <si>
+    <t>480.508 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063502165_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 90 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 09:21 AM</t>
+  </si>
+  <si>
+    <t>716.934 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063502165_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 89 [Elec]</t>
+  </si>
+  <si>
+    <t>1420.832 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063502165_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 88 [Elec]</t>
+  </si>
+  <si>
+    <t>4050.176 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063502165_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 38 [Elec]</t>
+  </si>
+  <si>
+    <t>515.631 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350168b_4</t>
+  </si>
+  <si>
+    <t>Coral Cove B204 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 09:23 AM</t>
+  </si>
+  <si>
+    <t>1395.195 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350168b_3</t>
+  </si>
+  <si>
+    <t>Coral Cove B203 [Elec]</t>
+  </si>
+  <si>
+    <t>782.146 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350168b_2</t>
+  </si>
+  <si>
+    <t>Coral Cove B202 [Elec]</t>
+  </si>
+  <si>
+    <t>1091.438 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350168b_1</t>
+  </si>
+  <si>
+    <t>Coral Cove B201 [Elec]</t>
+  </si>
+  <si>
+    <t>762.027 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350128a_9</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 06</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:47 AM</t>
+  </si>
+  <si>
+    <t>64.789 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350128a_8</t>
+  </si>
+  <si>
+    <t>229.403 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350128a_7</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 07</t>
+  </si>
+  <si>
+    <t>297.46 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350128a_6</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 08</t>
+  </si>
+  <si>
+    <t>214.779 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350128a_5</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 09</t>
+  </si>
+  <si>
+    <t>69.021 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350128a_4</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 10</t>
+  </si>
+  <si>
+    <t>121.53 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350128a_3</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 11</t>
+  </si>
+  <si>
+    <t>246.416 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350128a_2</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 12</t>
+  </si>
+  <si>
+    <t>70.824 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350128a_1</t>
+  </si>
+  <si>
+    <t>Coral Cove FF DB 13</t>
+  </si>
+  <si>
+    <t>94.24 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635003ed_5</t>
+  </si>
+  <si>
+    <t>Coral Cove A205 [Elec]</t>
+  </si>
+  <si>
+    <t>853.199 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635003ed_4</t>
+  </si>
+  <si>
+    <t>Coral Cove A204 [Elec]</t>
+  </si>
+  <si>
+    <t>479.548 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635003ed_3</t>
+  </si>
+  <si>
+    <t>Coral Cove A203 [Elec]</t>
+  </si>
+  <si>
+    <t>806.276 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635003ed_2</t>
+  </si>
+  <si>
+    <t>Coral Cove A202 [Elec]</t>
+  </si>
+  <si>
+    <t>1082.525 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635003ed_1</t>
+  </si>
+  <si>
+    <t>Coral Cove A201 [Elec]</t>
+  </si>
+  <si>
+    <t>1118.897 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635002db_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 74 [Elec]</t>
+  </si>
+  <si>
+    <t>341.986 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120635002db_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 73 [Elec]</t>
+  </si>
+  <si>
+    <t>1754.658 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350013b_7</t>
+  </si>
+  <si>
+    <t>Coral Cove 201 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:46 AM</t>
+  </si>
+  <si>
+    <t>957.882 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350013b_6</t>
+  </si>
+  <si>
+    <t>Coral Cove 197 [Elec]</t>
+  </si>
+  <si>
+    <t>9/22/2026, 02:55 PM</t>
+  </si>
+  <si>
+    <t>21.937 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350013b_5</t>
+  </si>
+  <si>
+    <t>Coral Cove 195 [Elec]</t>
+  </si>
+  <si>
+    <t>9/22/2026, 03:55 PM</t>
+  </si>
+  <si>
+    <t>49.245 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350013b_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 194 [Elec]</t>
+  </si>
+  <si>
+    <t>9/22/2026, 09:00 AM</t>
+  </si>
+  <si>
+    <t>15.868 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350013b_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 184 [Elec]</t>
+  </si>
+  <si>
+    <t>1223.817 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350013b_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 180 [Elec]</t>
+  </si>
+  <si>
+    <t>344.331 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206350013b_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 179 [Elec]</t>
+  </si>
+  <si>
+    <t>36.685 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063400e34_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 205 [Elec]</t>
+  </si>
+  <si>
+    <t>7/24/2026, 02:06 PM</t>
+  </si>
+  <si>
+    <t>97.136 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063400e34_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 204 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:28 AM</t>
+  </si>
+  <si>
+    <t>133.352 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063400e34_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 203 [Elec]</t>
+  </si>
+  <si>
+    <t>2400.102 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063400e34_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 202 [Elec]</t>
+  </si>
+  <si>
+    <t>123.528 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f120634007d5</t>
+  </si>
+  <si>
+    <t>Coral Cove MS5 Bulk [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:50 AM</t>
+  </si>
+  <si>
+    <t>453739.036 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f1206340076e</t>
+  </si>
+  <si>
+    <t>Coral Cove MS4 Bulk [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:43 AM</t>
+  </si>
+  <si>
+    <t>28448.196 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063102063_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 110 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:32 AM</t>
+  </si>
+  <si>
+    <t>1197.22 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063102063_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 109 [Elec]</t>
+  </si>
+  <si>
+    <t>10/7/2026, 11:16 AM</t>
+  </si>
+  <si>
+    <t>3804.691 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063102063_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 108 [Elec]</t>
+  </si>
+  <si>
+    <t>1683.597 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063102063_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 107 [Elec]</t>
+  </si>
+  <si>
+    <t>4775.081 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063101c2a_5</t>
+  </si>
+  <si>
+    <t>Coral Cove 94 [Elec]</t>
+  </si>
+  <si>
+    <t>4766.03 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063101c2a_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 98 [Elec]</t>
+  </si>
+  <si>
+    <t>2634.997 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063101c2a_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 97 [Elec]</t>
+  </si>
+  <si>
+    <t>4687.238 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063101c2a_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 96 [Elec]</t>
+  </si>
+  <si>
+    <t>3728.227 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063101c2a_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 95 [Elec]</t>
+  </si>
+  <si>
+    <t>4293.829 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063101a76_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 93 [Elec]</t>
+  </si>
+  <si>
+    <t>2792.975 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063101a76_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 92 [Elec]</t>
+  </si>
+  <si>
+    <t>682.169 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063101a76_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 91 [Elec]</t>
+  </si>
+  <si>
+    <t>2656.534 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063100f76_4</t>
+  </si>
+  <si>
+    <t>Coral Cove 102 [Elec]</t>
+  </si>
+  <si>
+    <t>10/9/2026, 08:42 AM</t>
+  </si>
+  <si>
+    <t>5234.448 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063100f76_3</t>
+  </si>
+  <si>
+    <t>Coral Cove 101 [Elec]</t>
+  </si>
+  <si>
+    <t>3195.848 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063100f76_2</t>
+  </si>
+  <si>
+    <t>Coral Cove 100 [Elec]</t>
+  </si>
+  <si>
+    <t>5388.593 kWh</t>
+  </si>
+  <si>
+    <t>2cf7f12063100f76_1</t>
+  </si>
+  <si>
+    <t>Coral Cove 99 [Elec]</t>
+  </si>
+  <si>
+    <t>3100.931 kWh</t>
   </si>
 </sst>
 </file>
@@ -1149,17 +2217,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3F792EA-E684-4376-A2DA-AE70FBFB7A6E}">
-  <dimension ref="A1:E68"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E177"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1176,7 +2244,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1193,7 +2261,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1210,7 +2278,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1227,7 +2295,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -1244,7 +2312,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1261,7 +2329,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>26</v>
       </c>
@@ -1278,7 +2346,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>30</v>
       </c>
@@ -1295,7 +2363,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>34</v>
       </c>
@@ -1312,7 +2380,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
@@ -1329,7 +2397,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
         <v>42</v>
       </c>
@@ -1346,7 +2414,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>46</v>
       </c>
@@ -1363,7 +2431,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
         <v>50</v>
       </c>
@@ -1380,7 +2448,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>54</v>
       </c>
@@ -1397,7 +2465,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>58</v>
       </c>
@@ -1414,7 +2482,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
         <v>62</v>
       </c>
@@ -1431,7 +2499,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
         <v>66</v>
       </c>
@@ -1448,7 +2516,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>69</v>
       </c>
@@ -1465,7 +2533,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>72</v>
       </c>
@@ -1482,7 +2550,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
         <v>75</v>
       </c>
@@ -1499,7 +2567,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
         <v>78</v>
       </c>
@@ -1516,7 +2584,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>81</v>
       </c>
@@ -1533,7 +2601,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
         <v>84</v>
       </c>
@@ -1550,7 +2618,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>87</v>
       </c>
@@ -1567,7 +2635,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>90</v>
       </c>
@@ -1584,7 +2652,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
         <v>93</v>
       </c>
@@ -1601,7 +2669,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
         <v>96</v>
       </c>
@@ -1618,7 +2686,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
         <v>99</v>
       </c>
@@ -1635,7 +2703,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
         <v>103</v>
       </c>
@@ -1652,7 +2720,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
         <v>106</v>
       </c>
@@ -1669,7 +2737,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
         <v>109</v>
       </c>
@@ -1686,7 +2754,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
         <v>112</v>
       </c>
@@ -1703,7 +2771,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
         <v>115</v>
       </c>
@@ -1720,7 +2788,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
         <v>118</v>
       </c>
@@ -1737,7 +2805,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
         <v>121</v>
       </c>
@@ -1754,7 +2822,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
         <v>124</v>
       </c>
@@ -1771,7 +2839,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
         <v>128</v>
       </c>
@@ -1788,7 +2856,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
         <v>132</v>
       </c>
@@ -1805,7 +2873,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
         <v>135</v>
       </c>
@@ -1822,7 +2890,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
         <v>138</v>
       </c>
@@ -1839,7 +2907,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
         <v>141</v>
       </c>
@@ -1856,7 +2924,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
         <v>144</v>
       </c>
@@ -1873,7 +2941,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
         <v>147</v>
       </c>
@@ -1890,7 +2958,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
         <v>150</v>
       </c>
@@ -1907,7 +2975,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
         <v>153</v>
       </c>
@@ -1924,7 +2992,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
         <v>156</v>
       </c>
@@ -1941,7 +3009,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
         <v>159</v>
       </c>
@@ -1958,7 +3026,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
         <v>162</v>
       </c>
@@ -1975,7 +3043,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
         <v>166</v>
       </c>
@@ -1992,7 +3060,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
         <v>170</v>
       </c>
@@ -2009,7 +3077,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
         <v>174</v>
       </c>
@@ -2026,7 +3094,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
         <v>177</v>
       </c>
@@ -2043,7 +3111,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
         <v>181</v>
       </c>
@@ -2060,7 +3128,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
         <v>184</v>
       </c>
@@ -2077,7 +3145,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
         <v>187</v>
       </c>
@@ -2094,7 +3162,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
         <v>190</v>
       </c>
@@ -2111,7 +3179,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
         <v>193</v>
       </c>
@@ -2128,7 +3196,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
         <v>196</v>
       </c>
@@ -2145,7 +3213,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
         <v>199</v>
       </c>
@@ -2162,7 +3230,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
         <v>203</v>
       </c>
@@ -2179,7 +3247,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
         <v>207</v>
       </c>
@@ -2196,7 +3264,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
         <v>210</v>
       </c>
@@ -2213,7 +3281,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
         <v>213</v>
       </c>
@@ -2230,7 +3298,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
         <v>216</v>
       </c>
@@ -2247,7 +3315,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A65" s="2" t="s">
         <v>219</v>
       </c>
@@ -2264,7 +3332,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A66" s="2" t="s">
         <v>222</v>
       </c>
@@ -2281,7 +3349,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
         <v>225</v>
       </c>
@@ -2298,7 +3366,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A68" s="2" t="s">
         <v>228</v>
       </c>
@@ -2313,6 +3381,1859 @@
       </c>
       <c r="E68" s="2" t="s">
         <v>230</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A69" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C69" s="2">
+        <v>91546269</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A70" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="C70" s="2">
+        <v>91546273</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A71" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C71" s="2">
+        <v>91546272</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A72" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C72" s="2">
+        <v>91546290</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A73" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C73" s="2">
+        <v>91546265</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A74" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C74" s="2">
+        <v>91732544</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A75" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C75" s="2">
+        <v>91732601</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A76" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C76" s="2">
+        <v>91732580</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A77" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C77" s="2">
+        <v>91733009</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A78" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C78" s="2">
+        <v>91732508</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A79" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C79" s="2">
+        <v>91546231</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A80" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C80" s="2">
+        <v>91546174</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A81" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C81" s="2">
+        <v>91733045</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A82" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C82" s="2">
+        <v>91733032</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A83" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C83" s="2">
+        <v>91732634</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A84" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C84" s="2">
+        <v>91732633</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A85" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C85" s="2">
+        <v>91732630</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A86" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C86" s="2">
+        <v>91732714</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A87" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C87" s="2">
+        <v>91732851</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A88" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C88" s="2">
+        <v>91732887</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A89" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C89" s="2">
+        <v>91732938</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A90" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C90" s="2">
+        <v>91732859</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A91" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C91" s="2">
+        <v>91732898</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A92" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A93" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="C93" s="2">
+        <v>91732661</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A94" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C94" s="2">
+        <v>91732631</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A95" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C95" s="2">
+        <v>91732654</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A96" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="C96" s="2">
+        <v>91732635</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A97" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C97" s="2">
+        <v>91732585</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A98" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C98" s="2">
+        <v>91732567</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A99" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="C99" s="2">
+        <v>91732512</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A100" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="C100" s="2">
+        <v>91732689</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A101" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="C101" s="2">
+        <v>91732713</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A102" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="C102" s="2">
+        <v>91732687</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A103" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="C103" s="2">
+        <v>91732662</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A104" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C104" s="2">
+        <v>91732642</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A105" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="C105" s="2">
+        <v>91732982</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A106" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="C106" s="2">
+        <v>91733051</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A107" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="C107" s="2">
+        <v>91733028</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A108" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C108" s="2">
+        <v>91733079</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A109" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C109" s="2">
+        <v>91733024</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A110" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="C110" s="2">
+        <v>91733073</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A111" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="C111" s="2">
+        <v>91733029</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A112" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="C112" s="2">
+        <v>91733031</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A113" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C113" s="2">
+        <v>91733022</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A114" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="C114" s="2">
+        <v>91732608</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A115" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C115" s="2">
+        <v>91732627</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A116" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="C116" s="2">
+        <v>91732604</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A117" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="C117" s="2">
+        <v>91732632</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A118" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="C118" s="2">
+        <v>91732606</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A119" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="C119" s="2">
+        <v>91732622</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A120" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="C120" s="2">
+        <v>91732626</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A121" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="C121" s="2">
+        <v>91732568</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A122" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C122" s="2">
+        <v>91732572</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A123" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="C123" s="2">
+        <v>91732556</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A124" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C124" s="2">
+        <v>91732548</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A125" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="C125" s="2">
+        <v>91732583</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A126" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="C126" s="2">
+        <v>91732584</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A127" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="C127" s="2">
+        <v>91732521</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A128" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C128" s="2">
+        <v>91732547</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A129" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="C129" s="2">
+        <v>91732609</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A130" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="C130" s="2">
+        <v>91732712</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A131" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C131" s="2">
+        <v>91732629</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A132" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="C132" s="2">
+        <v>91732690</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A133" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C133" s="2">
+        <v>91733075</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A134" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C134" s="2">
+        <v>91732873</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A135" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="C135" s="2">
+        <v>91732860</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A136" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="C136" s="2">
+        <v>91732856</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A137" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C137" s="2">
+        <v>91732875</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A138" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C138" s="2">
+        <v>91732876</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A139" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="C139" s="2">
+        <v>91732913</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A140" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="C140" s="2">
+        <v>91732886</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A141" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="C141" s="2">
+        <v>91732902</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A142" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="C142" s="2">
+        <v>91732688</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A143" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="C143" s="2">
+        <v>91732637</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A144" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="C144" s="2">
+        <v>91732636</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A145" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="C145" s="2">
+        <v>91732658</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A146" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="C146" s="2">
+        <v>91732614</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A147" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="C147" s="2">
+        <v>91732543</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A148" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="C148" s="2">
+        <v>91732539</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A149" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C149" s="2">
+        <v>91546259</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A150" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C150" s="2">
+        <v>91546320</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A151" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="C151" s="2">
+        <v>91546245</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A152" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C152" s="2">
+        <v>91546247</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A153" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="C153" s="2">
+        <v>91546191</v>
+      </c>
+      <c r="D153" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A154" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="C154" s="2">
+        <v>91733074</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A155" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="C155" s="2">
+        <v>91546193</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A156" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="C156" s="2">
+        <v>91732909</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A157" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="C157" s="2">
+        <v>91732885</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A158" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="C158" s="2">
+        <v>91732883</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="E158" s="2" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A159" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C159" s="2">
+        <v>91732870</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A160" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="C160" s="2">
+        <v>91074243</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="E160" s="2" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A161" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="C161" s="2">
+        <v>90915109</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="E161" s="2" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A162" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="C162" s="2">
+        <v>91732611</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E162" s="2" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A163" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="C163" s="2">
+        <v>91732561</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="E163" s="2" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A164" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="C164" s="2">
+        <v>91732651</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E164" s="2" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A165" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="C165" s="2">
+        <v>91732647</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E165" s="2" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A166" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="C166" s="2">
+        <v>91732613</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A167" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="C167" s="2">
+        <v>91732615</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A168" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="B168" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="C168" s="2">
+        <v>91732640</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E168" s="2" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A169" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="C169" s="2">
+        <v>91732641</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E169" s="2" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A170" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="B170" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C170" s="2">
+        <v>91732603</v>
+      </c>
+      <c r="D170" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E170" s="2" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A171" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B171" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="C171" s="2">
+        <v>91732666</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="E171" s="2" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A172" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="C172" s="2">
+        <v>91732605</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="E172" s="2" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A173" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="C173" s="2">
+        <v>91732665</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="E173" s="2" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A174" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="C174" s="2">
+        <v>91732607</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A175" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="B175" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="C175" s="2">
+        <v>91732610</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="E175" s="2" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A176" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="C176" s="2">
+        <v>91732638</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="E176" s="2" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A177" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="C177" s="2">
+        <v>91732612</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="E177" s="2" t="s">
+        <v>586</v>
       </c>
     </row>
   </sheetData>

</xml_diff>